<commit_message>
Actualización automática 2026-09-14 09:30:18
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -2313,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0</v>
+        <v>7495.2</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
@@ -2340,7 +2340,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>0</v>
+        <v>6982.18</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -2366,52 +2366,52 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
+          <t>1 de 30</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
           <t>0 de 30</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>0 de 30</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>0 de 30</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>1 de 30</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>0 de 30</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>0 de 30</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
         <is>
           <t>1 de 30</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="M32" s="4" t="inlineStr">
         <is>
           <t>1 de 30</t>
-        </is>
-      </c>
-      <c r="M32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
@@ -3223,7 +3223,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>14477.38</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>10000</v>
@@ -3240,7 +3240,7 @@
         <v>11295.33</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>1113.1</v>
+        <v>15590.48</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>38500</v>
@@ -3263,9 +3263,9 @@
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3339,13 +3339,13 @@
         <v>3800</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>7495.2</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3800</v>
+        <v>-3695.2</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>1.972421052631579</v>
       </c>
     </row>
     <row r="4">
@@ -3603,13 +3603,13 @@
         <v>39283</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>-71.11</v>
+        <v>6911.07</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>39354.11</v>
+        <v>32371.93</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.001810197795484052</v>
+        <v>0.1759303006389532</v>
       </c>
     </row>
     <row r="15">
@@ -3646,13 +3646,13 @@
         <v>50564.443</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1440.87</v>
+        <v>15918.25</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>49123.573</v>
+        <v>34646.193</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.02849571585313419</v>
+        <v>0.3148111411016631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-07 13:30:14
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1113,7 +1113,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>3780.48</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>0</v>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>0 de 30</t>
+          <t>1 de 30</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -2737,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>3780.48</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>1000</v>
@@ -3240,7 +3240,7 @@
         <v>42787.96</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>0</v>
+        <v>3780.48</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>38500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-19 08:30:16
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>NIZA ARIAS YOSELIN EDITH</t>
+          <t>TAMAYO VILLACIS EDWIN XAVIER</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TAMAYO VILLACIS EDWIN XAVIER</t>
+          <t>TOSCANO RAMIREZ MONICA CECILIA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TOSCANO RAMIREZ MONICA CECILIA</t>
+          <t>VARIEDADES-PAS SAS</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>VARIEDADES-PAS SAS</t>
+          <t>VELASQUEZ ARELLANO SAIRA MAGDALENA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>VELASQUEZ ARELLANO SAIRA MAGDALENA</t>
+          <t>VIDAL VARGAS ANDREA DOMINIQUE</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>VIDAL VARGAS ANDREA DOMINIQUE</t>
+          <t>ZAMBRANO ANGELA MARIA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2299,144 +2299,84 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>RIOS CARRION ANGEL BENIGNO</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>ZAMBRANO ANGELA MARIA</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>1 de 30</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="M32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="O32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="P32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="Q32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
-        </is>
-      </c>
-      <c r="R32" s="4" t="inlineStr">
-        <is>
-          <t>0 de 30</t>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
+        </is>
+      </c>
+      <c r="R31" s="4" t="inlineStr">
+        <is>
+          <t>0 de 29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-21 12:30:17
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1425,7 +1425,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>0</v>
+        <v>-95.7</v>
       </c>
       <c r="I16" s="2" t="n">
         <v>0</v>
@@ -2785,7 +2785,7 @@
         <v>3521.1</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>-95.7</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>4000</v>
@@ -3180,7 +3180,7 @@
         <v>42787.96</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>3780.48</v>
+        <v>3684.78</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>38500</v>
@@ -3205,7 +3205,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3375,13 +3375,13 @@
         <v>210</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>-95.7</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>210</v>
+        <v>305.7</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>-0.4557142857142857</v>
       </c>
     </row>
     <row r="8">
@@ -3586,13 +3586,13 @@
         <v>46882.053</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>3780.48</v>
+        <v>3684.78</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>43101.573</v>
+        <v>43197.273</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.08063810686788823</v>
+        <v>0.07859681400897696</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 10:30:18
</commit_message>
<xml_diff>
--- a/data/RIOS CARRION ANGEL BENIGNO.xlsx
+++ b/data/RIOS CARRION ANGEL BENIGNO.xlsx
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>0</v>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>0 de 29</t>
+          <t>1 de 29</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
@@ -3001,7 +3001,7 @@
         <v>17719.9</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -3180,7 +3180,7 @@
         <v>42787.96</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>3684.78</v>
+        <v>3702.69</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>38500</v>
@@ -3471,13 +3471,13 @@
         <v>203.763</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>203.763</v>
+        <v>185.853</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>0.0878962323876268</v>
       </c>
     </row>
     <row r="12">
@@ -3586,13 +3586,13 @@
         <v>46882.053</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>3684.78</v>
+        <v>3702.69</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>43197.273</v>
+        <v>43179.363</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.07859681400897696</v>
+        <v>0.0789788365283406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>